<commit_message>
docs: fault-check limitations and a description of every installation method
- Report limitations: the k^2 S^2 >= I^2t let-through check for devices faster than 0.1 s
  or current-limiting is not calculated; the fault pair entered must be the worst one
  along the cable (IS 732 clause 4.4.5.5.2).
- Template Guide sheet: a short description of each installation method (A1 to D2) and
  the grouping row the tool applies, from IS 732 Tables 19, 20, 36-38 and clause S-6.1.
- SOURCES.md: method codes checked item by item against IEC Table A.52.3; the same in both.
- Sample input and report regenerated.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/samples/sample-input.xlsx
+++ b/samples/sample-input.xlsx
@@ -914,7 +914,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C19"/>
+  <dimension ref="A1:C29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1105,7 +1105,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Installation method: A1, A2, B1, B2, C, E, D1, D2. D1 = in buried ducts, D2 = direct in the ground.</t>
+          <t>Installation method: A1, A2, B1, B2, C, E, D1, D2. Each is described in the Installation methods list below.</t>
         </is>
       </c>
     </row>
@@ -1242,6 +1242,123 @@
       <c r="C19" t="inlineStr">
         <is>
           <t>D1 and D2 only. Leave blank for 2.5.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Installation methods</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr"/>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Where the cable runs, and the grouping factors used</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr"/>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Single-core cables or insulated conductors in conduit in a thermally insulated wall. Grouping: bunched or enclosed (Table 36 item 1).</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>A2</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr"/>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Multi-core cable in conduit in a thermally insulated wall. Grouping: bunched or enclosed (Table 36 item 1).</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>B1</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr"/>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Single-core cables or insulated conductors in conduit or trunking on a wall, less than 0.3 x conduit diameter from it. Grouping: bunched or enclosed (Table 36 item 1).</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>B2</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr"/>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Multi-core cable in conduit on a wall, less than 0.3 x conduit diameter from it. Grouping: bunched or enclosed (Table 36 item 1).</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr"/>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Single-core or multi-core cable fixed on a wall, less than 0.3 x cable diameter from it; also used for cable on unperforated tray and cable direct in masonry. Grouping: single layer on wall, floor or unperforated tray (Table 36 item 2).</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr"/>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Multi-core cable in free air, at least 0.3 x cable diameter clear of any surface, for example on perforated tray, brackets or ladder. Grouping: single layer on perforated tray (Table 36 item 4).</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>D1</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr"/>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Multi-core cable in ducts in the ground (reference: 100 mm duct, 0.7 m deep). Grouping: ducts touching (Table 38).</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>D2</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr"/>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Cable laid direct in the ground (reference: 0.7 m deep). Grouping: cables touching (Table 37).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: cable construction drop-down replaces the cores column
Manas's own test entered cores = 1 meaning single-core cables; the tool meant loaded
conductors and stopped with an engine error that named no row (spec Rev3).

- Input: `cable` drop-down (2 x 1C, 3 x 1C, 4 x 1C, 2C, 3C, 3.5C, 4C). Loaded conductors
  come from phase (IS 732 clause 5.2.6.6.1). Refused, by row: cable/phase mismatch,
  single-core with method E (F/G not covered) and with A2 (use A1).
- Every engine error is reported as Row n (tag), all cables at once.
- Report: heading and summary show the construction; limitation lines for parallel runs,
  F/G, and the 3.5C reduced neutral.
- Worked examples gain a cable value; no calculated value changes.
- README gains the fault-check limitations missed in PR #12. Samples regenerated.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/samples/sample-input.xlsx
+++ b/samples/sample-input.xlsx
@@ -550,7 +550,7 @@
       </c>
       <c r="K1" t="inlineStr">
         <is>
-          <t>cores</t>
+          <t>cable</t>
         </is>
       </c>
       <c r="L1" t="inlineStr">
@@ -627,8 +627,10 @@
           <t>C</t>
         </is>
       </c>
-      <c r="K2" t="n">
-        <v>3</v>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>3C</t>
+        </is>
       </c>
       <c r="L2" t="n">
         <v>40</v>
@@ -687,8 +689,10 @@
           <t>B1</t>
         </is>
       </c>
-      <c r="K3" t="n">
-        <v>2</v>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>2 x 1C</t>
+        </is>
       </c>
       <c r="L3" t="n">
         <v>35</v>
@@ -747,8 +751,10 @@
           <t>E</t>
         </is>
       </c>
-      <c r="K4" t="n">
-        <v>3</v>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>4C</t>
+        </is>
       </c>
       <c r="L4" t="n">
         <v>30</v>
@@ -807,8 +813,10 @@
           <t>D2</t>
         </is>
       </c>
-      <c r="K5" t="n">
-        <v>3</v>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>3.5C</t>
+        </is>
       </c>
       <c r="L5" t="n">
         <v>30</v>
@@ -867,8 +875,10 @@
           <t>C</t>
         </is>
       </c>
-      <c r="K6" t="n">
-        <v>3</v>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>4 x 1C</t>
+        </is>
       </c>
       <c r="L6" t="n">
         <v>40</v>
@@ -890,7 +900,7 @@
       </c>
     </row>
   </sheetData>
-  <dataValidations count="4">
+  <dataValidations count="5">
     <dataValidation sqref="B2:B500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"1ph,3ph"</formula1>
     </dataValidation>
@@ -902,6 +912,9 @@
     </dataValidation>
     <dataValidation sqref="J2:J500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"A1,A2,B1,B2,C,E,D1,D2"</formula1>
+    </dataValidation>
+    <dataValidation sqref="K2:K500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"2 x 1C,3 x 1C,4 x 1C,2C,3C,3.5C,4C"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1112,7 +1125,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>cores</t>
+          <t>cable</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1122,7 +1135,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>LOADED conductors: 2 for 1ph, 3 for 3ph (a 4-core 3ph cable is entered as 3).</t>
+          <t>Cable construction: 2 x 1C or 2C (1ph); 3C (1ph or 3ph); 3 x 1C, 4 x 1C, 3.5C or 4C (3ph). n x 1C = n single-core cables. Single-core cables cannot use method E (free air is methods F and G, not covered) or A2 (use A1). For 3.5C the size is the phase conductor.</t>
         </is>
       </c>
     </row>
@@ -1251,7 +1264,6 @@
           <t>Installation methods</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr"/>
       <c r="C21" t="inlineStr">
         <is>
           <t>Where the cable runs, and the grouping factors used</t>
@@ -1264,7 +1276,6 @@
           <t>A1</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr"/>
       <c r="C22" t="inlineStr">
         <is>
           <t>Single-core cables or insulated conductors in conduit in a thermally insulated wall. Grouping: bunched or enclosed (Table 36 item 1).</t>
@@ -1277,7 +1288,6 @@
           <t>A2</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr">
         <is>
           <t>Multi-core cable in conduit in a thermally insulated wall. Grouping: bunched or enclosed (Table 36 item 1).</t>
@@ -1290,7 +1300,6 @@
           <t>B1</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr">
         <is>
           <t>Single-core cables or insulated conductors in conduit or trunking on a wall, less than 0.3 x conduit diameter from it. Grouping: bunched or enclosed (Table 36 item 1).</t>
@@ -1303,7 +1312,6 @@
           <t>B2</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr"/>
       <c r="C25" t="inlineStr">
         <is>
           <t>Multi-core cable in conduit on a wall, less than 0.3 x conduit diameter from it. Grouping: bunched or enclosed (Table 36 item 1).</t>
@@ -1316,7 +1324,6 @@
           <t>C</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr">
         <is>
           <t>Single-core or multi-core cable fixed on a wall, less than 0.3 x cable diameter from it; also used for cable on unperforated tray and cable direct in masonry. Grouping: single layer on wall, floor or unperforated tray (Table 36 item 2).</t>
@@ -1329,7 +1336,6 @@
           <t>E</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr">
         <is>
           <t>Multi-core cable in free air, at least 0.3 x cable diameter clear of any surface, for example on perforated tray, brackets or ladder. Grouping: single layer on perforated tray (Table 36 item 4).</t>
@@ -1342,7 +1348,6 @@
           <t>D1</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr"/>
       <c r="C28" t="inlineStr">
         <is>
           <t>Multi-core cable in ducts in the ground (reference: 100 mm duct, 0.7 m deep). Grouping: ducts touching (Table 38).</t>
@@ -1355,7 +1360,6 @@
           <t>D2</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr">
         <is>
           <t>Cable laid direct in the ground (reference: 0.7 m deep). Grouping: cables touching (Table 37).</t>

</xml_diff>